<commit_message>
qol: add Valkyrie and Papillon tactical role clarifications to class
add Valkyrie and Papillon tactical role clarifications to class text

- Valkyrie (ClassData_03.bin): clarify spear and sword weapons, front
line Circle Protection party defense, and counterattacks while retaining
war angel lore. - Papillon (ClassData_30.bin): add master of turn delay
/ tempo role while preserving hand-fans, dual-range capability, and the
food joke intact. - Dark Lord and Joker remain 100% vanilla as intended.
- Verified in build_variant.py qol (49 classes verified, 9 modified, 40
byte-identical) and full test suite (196/196 passing).
</commit_message>
<xml_diff>
--- a/mod_project/data_tables/qol_class_text.xlsx
+++ b/mod_project/data_tables/qol_class_text.xlsx
@@ -612,14 +612,14 @@
       </c>
       <c r="F5" t="inlineStr">
         <is>
-          <t>They have no superior when it comes to short-range fortitude. With their immense 
-strength and beauty, they are oft likened to war angels leading armies into battle.
-Their strong counterattack as they defend their allies seals the victory.</t>
+          <t>They have no superior when it comes to short-range fortitude. Wielding spears
+and swords, these war angels guard the front line with Circle Protection, shielding
+the entire party from physical assaults while executing swift counterattacks.</t>
         </is>
       </c>
       <c r="G5" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H5" t="n">
@@ -1742,18 +1742,18 @@
       </c>
       <c r="F32" t="inlineStr">
         <is>
-          <t>Using hand-fans proficiently as weapons, they are skilled in both short and long 
-distance combat. They are unique not only in weapon choice, but also skill selection, 
-most notable of which is an ultimate skill that turns a weakened enemy into... food?</t>
+          <t>Using hand-fans proficiently as weapons, they are skilled in both short and long
+distance combat. Masters of turn delay, they boast unique skills, not least of which
+is an ultimate skill that turns a weakened enemy into... food?</t>
         </is>
       </c>
       <c r="G32" t="inlineStr">
         <is>
-          <t>No</t>
+          <t>Yes</t>
         </is>
       </c>
       <c r="H32" t="n">
-        <v>86</v>
+        <v>84</v>
       </c>
     </row>
     <row r="33">

</xml_diff>